<commit_message>
[feat/HD-15447] Normalized Formatting in GeneXpert TB Workload report
</commit_message>
<xml_diff>
--- a/api/templates/genxpert_tb_workload_report/fr.xlsx
+++ b/api/templates/genxpert_tb_workload_report/fr.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10309"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/harshthakkar/Desktop/Projects/aspect/api/templates/genxpert_tb_workload_report/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahernandez/repos/aspect/api/templates/genxpert_tb_workload_report/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3E1AAC67-E128-2A4A-82F3-B96AB767D9A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9686B9B-B6A5-4642-AC00-A8ED20EEB1EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Devices" sheetId="1" r:id="rId1"/>
+    <sheet name="Appareils" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -324,54 +324,32 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm"/>
-    <numFmt numFmtId="165" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color indexed="64"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b/>
-      <sz val="16"/>
-      <color indexed="64"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="12"/>
-      <color indexed="64"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="12"/>
-      <color indexed="64"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color indexed="64"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="16"/>
+      <color indexed="64"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
       <color indexed="64"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -384,13 +362,7 @@
       <family val="2"/>
     </font>
     <font>
-      <u/>
-      <sz val="12"/>
-      <color indexed="64"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
+      <b/>
       <sz val="12"/>
       <color indexed="64"/>
       <name val="Calibri"/>
@@ -399,6 +371,12 @@
     <font>
       <b/>
       <sz val="12"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color indexed="64"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -417,7 +395,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -441,41 +419,13 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color auto="1"/>
       </left>
       <right style="thin">
         <color auto="1"/>
       </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
+      <top/>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
@@ -485,68 +435,63 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="11" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -781,33 +726,41 @@
     <col min="2" max="2" width="30.6640625" customWidth="1"/>
     <col min="3" max="3" width="35.33203125" customWidth="1"/>
     <col min="4" max="4" width="33.5" customWidth="1"/>
-    <col min="5" max="8" width="15.33203125" customWidth="1"/>
-    <col min="9" max="11" width="11.6640625" customWidth="1"/>
-    <col min="12" max="13" width="15.6640625" customWidth="1"/>
-    <col min="14" max="14" width="24.5" customWidth="1"/>
-    <col min="15" max="16" width="11.6640625" customWidth="1"/>
-    <col min="17" max="24" width="15.6640625" customWidth="1"/>
-    <col min="25" max="27" width="20.6640625" customWidth="1"/>
+    <col min="5" max="5" width="28.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.33203125" customWidth="1"/>
+    <col min="8" max="8" width="17.83203125" customWidth="1"/>
+    <col min="9" max="10" width="11.6640625" customWidth="1"/>
+    <col min="11" max="11" width="12.5" customWidth="1"/>
+    <col min="12" max="12" width="11" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.6640625" customWidth="1"/>
+    <col min="14" max="14" width="13.5" customWidth="1"/>
+    <col min="15" max="15" width="10.83203125" customWidth="1"/>
+    <col min="16" max="16" width="11.33203125" customWidth="1"/>
+    <col min="17" max="17" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.5" customWidth="1"/>
+    <col min="24" max="24" width="16" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="26" max="27" width="20.6640625" customWidth="1"/>
     <col min="28" max="28" width="20.6640625" style="1" customWidth="1"/>
     <col min="29" max="29" width="20.1640625" style="1" customWidth="1"/>
     <col min="30" max="30" width="33.33203125" customWidth="1"/>
     <col min="31" max="32" width="25.6640625" customWidth="1"/>
-    <col min="33" max="33" width="20.6640625" customWidth="1"/>
-    <col min="34" max="34" width="21.1640625" bestFit="1"/>
-    <col min="35" max="35" width="19" bestFit="1"/>
-    <col min="36" max="36" width="20.33203125" bestFit="1"/>
-    <col min="37" max="37" width="16.83203125" bestFit="1"/>
-    <col min="38" max="38" width="16.6640625" bestFit="1"/>
-    <col min="39" max="39" width="18.1640625" bestFit="1"/>
-    <col min="40" max="40" width="22" bestFit="1"/>
-    <col min="41" max="41" width="24.33203125" bestFit="1"/>
-    <col min="42" max="42" width="14.83203125" bestFit="1"/>
-    <col min="43" max="43" width="29.1640625" bestFit="1"/>
-    <col min="44" max="44" width="48.6640625" customWidth="1"/>
+    <col min="33" max="33" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="21.1640625" customWidth="1"/>
+    <col min="35" max="35" width="20.6640625" customWidth="1"/>
+    <col min="36" max="36" width="20.33203125" customWidth="1"/>
+    <col min="37" max="37" width="16.83203125" customWidth="1"/>
+    <col min="38" max="38" width="16.6640625" customWidth="1"/>
+    <col min="39" max="39" width="18.1640625" customWidth="1"/>
+    <col min="40" max="40" width="22" customWidth="1"/>
+    <col min="41" max="41" width="24.33203125" customWidth="1"/>
+    <col min="42" max="42" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="43" max="44" width="29.1640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:44" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="2" t="s">
         <v>59</v>
       </c>
       <c r="C1" s="2"/>
@@ -829,11 +782,11 @@
       <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="21" t="s">
+      <c r="C3" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -847,23 +800,23 @@
       <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="22" t="s">
+      <c r="C5" s="3" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="6" spans="1:44" ht="50.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C6" s="23" t="s">
+      <c r="C6" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="D6" s="24" t="s">
+      <c r="D6" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="E6" s="19"/>
-      <c r="F6" s="19"/>
-      <c r="G6" s="19"/>
-      <c r="H6" s="19"/>
-      <c r="I6" s="19"/>
-      <c r="J6" s="19"/>
+      <c r="E6" s="12"/>
+      <c r="F6" s="12"/>
+      <c r="G6" s="12"/>
+      <c r="H6" s="12"/>
+      <c r="I6" s="12"/>
+      <c r="J6" s="12"/>
     </row>
     <row r="7" spans="1:44" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="6"/>
@@ -871,34 +824,34 @@
     <row r="8" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A8" s="7"/>
     </row>
-    <row r="9" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:44" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:44" s="8" customFormat="1" ht="51" x14ac:dyDescent="0.2">
-      <c r="A10" s="25" t="s">
+    <row r="10" spans="1:44" s="8" customFormat="1" ht="52" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="B10" s="25" t="s">
+      <c r="B10" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="C10" s="25" t="s">
+      <c r="C10" s="9" t="s">
         <v>66</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="E10" s="25" t="s">
+      <c r="E10" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="F10" s="25" t="s">
+      <c r="F10" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="G10" s="25" t="s">
+      <c r="G10" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="H10" s="25" t="s">
+      <c r="H10" s="9" t="s">
         <v>70</v>
       </c>
       <c r="I10" s="9" t="s">
@@ -907,25 +860,25 @@
       <c r="J10" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="K10" s="25" t="s">
+      <c r="K10" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="L10" s="9" t="s">
+      <c r="L10" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="M10" s="9" t="s">
+      <c r="M10" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="N10" s="25" t="s">
+      <c r="N10" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="O10" s="26" t="s">
+      <c r="O10" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="P10" s="27" t="s">
+      <c r="P10" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="Q10" s="25" t="s">
+      <c r="Q10" s="14" t="s">
         <v>75</v>
       </c>
       <c r="R10" s="9" t="s">
@@ -946,215 +899,215 @@
       <c r="W10" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="X10" s="26" t="s">
+      <c r="X10" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="Y10" s="26" t="s">
+      <c r="Y10" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="Z10" s="25" t="s">
+      <c r="Z10" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="AA10" s="29" t="s">
+      <c r="AA10" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="AB10" s="28" t="s">
+      <c r="AB10" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="AC10" s="28" t="s">
+      <c r="AC10" s="16" t="s">
         <v>79</v>
       </c>
-      <c r="AD10" s="25" t="s">
+      <c r="AD10" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="AE10" s="25" t="s">
+      <c r="AE10" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="AF10" s="25" t="s">
+      <c r="AF10" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="AG10" s="30" t="s">
+      <c r="AG10" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="AH10" s="30" t="s">
+      <c r="AH10" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="AI10" s="30" t="s">
+      <c r="AI10" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="AJ10" s="30" t="s">
+      <c r="AJ10" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="AK10" s="30" t="s">
+      <c r="AK10" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="AL10" s="10" t="s">
+      <c r="AL10" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="AM10" s="30" t="s">
+      <c r="AM10" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="AN10" s="30" t="s">
+      <c r="AN10" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="AO10" s="30" t="s">
+      <c r="AO10" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="AP10" s="30" t="s">
+      <c r="AP10" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="AQ10" s="30" t="s">
+      <c r="AQ10" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="AR10" s="30" t="s">
+      <c r="AR10" s="9" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="11" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A11" s="11" t="s">
+      <c r="A11" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="D11" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="E11" s="11" t="s">
+      <c r="E11" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="F11" s="11" t="s">
+      <c r="F11" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="G11" s="11" t="s">
+      <c r="G11" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="H11" s="11" t="s">
+      <c r="H11" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="I11" s="11" t="s">
+      <c r="I11" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="J11" s="11" t="s">
+      <c r="J11" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="K11" s="11" t="s">
+      <c r="K11" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="L11" s="12" t="s">
+      <c r="L11" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="M11" s="12" t="s">
+      <c r="M11" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="N11" s="12" t="s">
+      <c r="N11" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="O11" s="11" t="s">
+      <c r="O11" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="P11" s="11" t="s">
+      <c r="P11" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="Q11" s="11" t="s">
+      <c r="Q11" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="R11" s="12" t="s">
+      <c r="R11" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="S11" s="12" t="s">
+      <c r="S11" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="T11" s="12" t="s">
+      <c r="T11" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="U11" s="12" t="s">
+      <c r="U11" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="V11" s="12" t="s">
+      <c r="V11" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="W11" s="12" t="s">
+      <c r="W11" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="X11" s="11" t="s">
+      <c r="X11" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="Y11" s="11" t="s">
+      <c r="Y11" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="Z11" s="11" t="s">
+      <c r="Z11" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="AA11" s="11" t="s">
+      <c r="AA11" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="AB11" s="13" t="e">
+      <c r="AB11" s="21" t="e">
         <f>IF(AG11=0,0,L11/AG11)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AC11" s="14" t="e">
+      <c r="AC11" s="22" t="e">
         <f>IF(AG11=0,0,(L11+M11)/AG11)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AD11" s="14" t="e">
+      <c r="AD11" s="22" t="e">
         <f>IF(AC11&gt;0.05,"High Rate of Errors/Invalids. Contact Lab.","")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AE11" s="14" t="s">
+      <c r="AE11" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="AF11" s="14" t="s">
+      <c r="AF11" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="AG11" s="11" t="s">
+      <c r="AG11" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="AH11" s="15" t="s">
+      <c r="AH11" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="AI11" s="16" t="s">
+      <c r="AI11" s="24" t="s">
         <v>49</v>
       </c>
-      <c r="AJ11" s="16" t="s">
+      <c r="AJ11" s="24" t="s">
         <v>50</v>
       </c>
-      <c r="AK11" s="16" t="s">
+      <c r="AK11" s="24" t="s">
         <v>51</v>
       </c>
-      <c r="AL11" s="16" t="s">
+      <c r="AL11" s="24" t="s">
         <v>52</v>
       </c>
-      <c r="AM11" s="16" t="s">
+      <c r="AM11" s="24" t="s">
         <v>53</v>
       </c>
-      <c r="AN11" s="16" t="s">
+      <c r="AN11" s="24" t="s">
         <v>54</v>
       </c>
-      <c r="AO11" s="15" t="s">
+      <c r="AO11" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="AP11" s="16" t="s">
+      <c r="AP11" s="25" t="s">
         <v>56</v>
       </c>
-      <c r="AQ11" s="16" t="s">
+      <c r="AQ11" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="AR11" s="16" t="s">
+      <c r="AR11" s="24" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="14" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="B14" s="17"/>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
-      <c r="G14" s="17"/>
-      <c r="H14" s="17"/>
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>